<commit_message>
Publica el deck de la Sesión 4 y construye sus scripts
Agrega el deck de la Sesión 4 (joins, pivots, NA y stringr) junto con el
guion de exposición y el bloque de práctica, que construye el ETL de la
EIGH y deja output/eigh_etl.rds como insumo de la Sesión 5.

El bloque de texto necesitaba material sucio sobre el cual trabajar: el
generador emite ahora una cuarta hoja en eigh_catalogos.xlsx con la clave
pegada a la etiqueta, separadores que cambian de fila en fila y
capitalización despareja. El regex de la sesión construye con ella la
llave que el join necesita, de modo que las dos mitades de la sesión se
encadenan en vez de quedar sueltas.

La semilla fija deja los CSV y el TXT byte a byte idénticos, así que las
salidas de las Sesiones 2 y 3 siguen vigentes; la única línea afectada es
el excel_sheets() de la Sesión 2, que ahora reporta cuatro hojas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYuZsEK575jHYXHF1vwoS3
</commit_message>
<xml_diff>
--- a/code/files/eigh_catalogos.xlsx
+++ b/code/files/eigh_catalogos.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="entidades" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="claves_gasto" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="notas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="rubros_texto" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="notas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t xml:space="preserve">Catálogo de entidades federativas</t>
   </si>
@@ -142,10 +143,58 @@
     <t xml:space="preserve">Ropa, calzado y accesorios</t>
   </si>
   <si>
+    <t xml:space="preserve">Clasificación del gasto - captura de campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rubro_completo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A001 - Alimentos consumidos dentro del hogar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">necesario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A002 – ALIMENTOS CONSUMIDOS FUERA DEL HOGAR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">discrecional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  B001- Renta o pago de vivienda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NECESARIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B002 : Electricidad,  agua y combustible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Necesario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C001 - transporte público y particular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D001  -  Colegiaturas y material escolar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">E001- CONSULTAS, medicamentos y hospitalización</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F001 – Ropa, calzado y accesorios  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discrecional</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notas metodológicas</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">1. Los montos son trimestrales y están expresados en pesos corrientes.</t>
@@ -680,13 +729,11 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>43</v>
-      </c>
-    </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" t="s">
         <v>44</v>
       </c>
     </row>
@@ -694,10 +741,100 @@
       <c r="A4" t="s">
         <v>45</v>
       </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>